<commit_message>
Cải modun sản lượng, sửa lỗi in lý lịch thiết bị/xe
</commit_message>
<xml_diff>
--- a/cung_cap_dl/kho_bao_tri/sl_mau_16.xlsx
+++ b/cung_cap_dl/kho_bao_tri/sl_mau_16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\kho_bao_tri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729788BE-EA98-46EB-B0B6-58F37EB0732C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E74917-1B1D-4E8F-80B6-D60A70736C55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>Ngày</t>
   </si>
@@ -77,6 +77,24 @@
   </si>
   <si>
     <t>Đội</t>
+  </si>
+  <si>
+    <t>2A2</t>
+  </si>
+  <si>
+    <t>5A2</t>
+  </si>
+  <si>
+    <t>5B2</t>
+  </si>
+  <si>
+    <t>7A2</t>
+  </si>
+  <si>
+    <t>7B2</t>
+  </si>
+  <si>
+    <t>9A2</t>
   </si>
 </sst>
 </file>
@@ -562,7 +580,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -626,7 +644,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -690,7 +708,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -754,7 +772,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -818,7 +836,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -882,7 +900,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>

</xml_diff>